<commit_message>
fixed crashes when closing excel fixed problem that selected executable was ignored several improvements to output
</commit_message>
<xml_diff>
--- a/test/testScriptAddin.xlsx
+++ b/test/testScriptAddin.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="28730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29328"/>
   <workbookPr codeName="DieseArbeitsmappe" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\dev\ScriptAddin\test\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C28F3EA1-21AD-41F2-A9F8-C9116DF7A99A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF16CAD5-1E25-45A7-A20A-EA0F5F0851D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17790" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17790" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Main Test" sheetId="1" r:id="rId1"/>
@@ -246,26 +246,6 @@
     <t>testdiagramperl</t>
   </si>
   <si>
-    <t>import matplotlib.pyplot as plt
-import numpy as np
-from inspect import getsourcefile
-from os.path import abspath, dirname
-from os import chdir
-print("changing to script dir..")
-scriptpath = dirname(abspath(getsourcefile(lambda:0)))
-chdir(scriptpath)
-print("loading data ..")
-csvfile = np.loadtxt('test_in.txt',skiprows=1,unpack=True)
-np.savetxt('test_out.txt',csvfile[1])
-print(csvfile[1],csvfile[2])
-print("plotting data ..")
-plt.scatter(csvfile[1],csvfile[2])
-plt.ylabel('in2')
-plt.xlabel('in1')
-plt.savefig("testdiagrampython.png", dpi=300, format='png')
-print("finished ..")</t>
-  </si>
-  <si>
     <t>var fs, infile;
 var in1 = new Array();
 var arrValues = new Array();
@@ -372,6 +352,32 @@
 binmode IMG;
 print IMG $gd-&gt;png;
 print "finished \n";</t>
+  </si>
+  <si>
+    <t>import matplotlib.pyplot as plt
+import numpy as np
+from inspect import getsourcefile
+from os.path import abspath, dirname
+from os import chdir
+import time
+print("changing to script dir..", flush=True)
+for i in range(100):
+  time.sleep(0.1)
+  print("loop "+str(i), flush=True)
+  if i%10 == 0:
+    print("-----------------&gt; "+str(i), flush=True)
+scriptpath = dirname(abspath(getsourcefile(lambda:0)))
+chdir(scriptpath)
+print("loading data ..", flush=True)
+csvfile = np.loadtxt('test_in.txt',skiprows=1,unpack=True)
+np.savetxt('test_out.txt',csvfile[1])
+print(csvfile[1],csvfile[2])
+print("plotting data ..", flush=True)
+plt.scatter(csvfile[1],csvfile[2])
+plt.ylabel('in2')
+plt.xlabel('in1')
+plt.savefig("testdiagrampython.png", dpi=300, format='png')
+print("finished ..", flush=True)</t>
   </si>
 </sst>
 </file>
@@ -581,6 +587,68 @@
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+      <xdr:twoCellAnchor editAs="oneCell">
+        <xdr:from>
+          <xdr:col>15</xdr:col>
+          <xdr:colOff>466725</xdr:colOff>
+          <xdr:row>6</xdr:row>
+          <xdr:rowOff>142875</xdr:rowOff>
+        </xdr:from>
+        <xdr:to>
+          <xdr:col>17</xdr:col>
+          <xdr:colOff>1238250</xdr:colOff>
+          <xdr:row>8</xdr:row>
+          <xdr:rowOff>123825</xdr:rowOff>
+        </xdr:to>
+        <xdr:sp macro="" textlink="">
+          <xdr:nvSpPr>
+            <xdr:cNvPr id="1025" name="Script_" hidden="1">
+              <a:extLst>
+                <a:ext uri="{63B3BB69-23CF-44E3-9099-C40C66FF867C}">
+                  <a14:compatExt spid="_x0000_s1025"/>
+                </a:ext>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000001040000}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvSpPr/>
+          </xdr:nvSpPr>
+          <xdr:spPr bwMode="auto">
+            <a:xfrm>
+              <a:off x="0" y="0"/>
+              <a:ext cx="0" cy="0"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:solidFill>
+              <a:srgbClr val="FFFFFF" mc:Ignorable="a14" a14:legacySpreadsheetColorIndex="65"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:extLst>
+              <a:ext uri="{91240B29-F687-4F45-9708-019B960494DF}">
+                <a14:hiddenLine w="9525">
+                  <a:solidFill>
+                    <a:srgbClr val="000000" mc:Ignorable="a14" a14:legacySpreadsheetColorIndex="64"/>
+                  </a:solidFill>
+                  <a:miter lim="800000"/>
+                  <a:headEnd/>
+                  <a:tailEnd/>
+                </a14:hiddenLine>
+              </a:ext>
+            </a:extLst>
+          </xdr:spPr>
+        </xdr:sp>
+        <xdr:clientData/>
+      </xdr:twoCellAnchor>
+    </mc:Choice>
+    <mc:Fallback/>
+  </mc:AlternateContent>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>9</xdr:col>
@@ -596,10 +664,10 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="7" name="testdiagram.png">
+        <xdr:cNvPr id="3" name="testdiagram.png">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{7B94FE94-97BC-4C15-8AFB-2454F504DEF6}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E7D46AC0-2896-9EAB-4DB9-A2325A3CB27D}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -631,79 +699,6 @@
     </xdr:pic>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
-      <xdr:twoCellAnchor editAs="oneCell">
-        <xdr:from>
-          <xdr:col>15</xdr:col>
-          <xdr:colOff>466724</xdr:colOff>
-          <xdr:row>6</xdr:row>
-          <xdr:rowOff>142875</xdr:rowOff>
-        </xdr:from>
-        <xdr:to>
-          <xdr:col>17</xdr:col>
-          <xdr:colOff>1238250</xdr:colOff>
-          <xdr:row>8</xdr:row>
-          <xdr:rowOff>123825</xdr:rowOff>
-        </xdr:to>
-        <xdr:sp macro="" textlink="">
-          <xdr:nvSpPr>
-            <xdr:cNvPr id="1025" name="Script_" hidden="1">
-              <a:extLst>
-                <a:ext uri="{63B3BB69-23CF-44E3-9099-C40C66FF867C}">
-                  <a14:compatExt spid="_x0000_s1025"/>
-                </a:ext>
-                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B6E6C0C6-00B8-1BF9-5011-E3478CF6F8ED}"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPr>
-            <xdr:cNvSpPr/>
-          </xdr:nvSpPr>
-          <xdr:spPr bwMode="auto">
-            <a:xfrm>
-              <a:off x="0" y="0"/>
-              <a:ext cx="0" cy="0"/>
-            </a:xfrm>
-            <a:prstGeom prst="rect">
-              <a:avLst/>
-            </a:prstGeom>
-            <a:solidFill>
-              <a:srgbClr val="FFFFFF" mc:Ignorable="a14" a14:legacySpreadsheetColorIndex="65"/>
-            </a:solidFill>
-            <a:ln>
-              <a:noFill/>
-            </a:ln>
-            <a:effectLst/>
-            <a:extLst>
-              <a:ext uri="{91240B29-F687-4F45-9708-019B960494DF}">
-                <a14:hiddenLine w="9525">
-                  <a:solidFill>
-                    <a:srgbClr val="000000" mc:Ignorable="a14" a14:legacySpreadsheetColorIndex="64"/>
-                  </a:solidFill>
-                  <a:prstDash val="solid"/>
-                  <a:miter lim="800000"/>
-                  <a:headEnd/>
-                  <a:tailEnd type="none" w="med" len="med"/>
-                </a14:hiddenLine>
-              </a:ext>
-              <a:ext uri="{AF507438-7753-43E0-B8FC-AC1667EBCBE1}">
-                <a14:hiddenEffects>
-                  <a:effectLst>
-                    <a:outerShdw dist="35921" dir="2700000" algn="ctr" rotWithShape="0">
-                      <a:srgbClr val="808080"/>
-                    </a:outerShdw>
-                  </a:effectLst>
-                </a14:hiddenEffects>
-              </a:ext>
-            </a:extLst>
-          </xdr:spPr>
-        </xdr:sp>
-        <xdr:clientData/>
-      </xdr:twoCellAnchor>
-    </mc:Choice>
-    <mc:Fallback/>
-  </mc:AlternateContent>
 </xdr:wsDr>
 </file>
 
@@ -829,15 +824,15 @@
     <xdr:to>
       <xdr:col>10</xdr:col>
       <xdr:colOff>518172</xdr:colOff>
-      <xdr:row>9</xdr:row>
+      <xdr:row>3</xdr:row>
       <xdr:rowOff>17154</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="3" name="testdiagrampython.png">
+        <xdr:cNvPr id="8" name="testdiagrampython.png">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5E85460C-52BD-45E1-BCA5-19EE7C3581EE}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{968D0E90-D5DA-3E11-91EB-C58600D7C694}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1280,7 +1275,7 @@
     </row>
     <row r="2" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A2" s="9">
-        <v>0.7</v>
+        <v>0.40250000000000002</v>
       </c>
       <c r="B2" s="9">
         <v>0.29749999999999999</v>
@@ -1305,33 +1300,33 @@
       </c>
       <c r="I2" s="3"/>
       <c r="J2" s="18" t="s">
+        <v>49</v>
+      </c>
+      <c r="K2" s="19" t="s">
         <v>50</v>
       </c>
-      <c r="K2" s="19" t="s">
-        <v>51</v>
-      </c>
       <c r="M2" s="18" t="s">
+        <v>49</v>
+      </c>
+      <c r="N2" s="19" t="s">
         <v>50</v>
       </c>
-      <c r="N2" s="19" t="s">
-        <v>51</v>
-      </c>
       <c r="P2" s="18" t="s">
+        <v>49</v>
+      </c>
+      <c r="Q2" s="19" t="s">
         <v>50</v>
       </c>
-      <c r="Q2" s="19" t="s">
-        <v>51</v>
-      </c>
       <c r="S2" s="18" t="s">
+        <v>49</v>
+      </c>
+      <c r="T2" s="19" t="s">
         <v>50</v>
-      </c>
-      <c r="T2" s="19" t="s">
-        <v>51</v>
       </c>
     </row>
     <row r="3" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A3" s="9">
-        <v>0.81410000000000005</v>
+        <v>0.50719999999999898</v>
       </c>
       <c r="B3" s="9">
         <v>0.30690000000000001</v>
@@ -1388,7 +1383,7 @@
     </row>
     <row r="4" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A4" s="9">
-        <v>2.75E-2</v>
+        <v>1.7100000000000001E-2</v>
       </c>
       <c r="B4" s="9">
         <v>1.04E-2</v>
@@ -1445,7 +1440,7 @@
     </row>
     <row r="5" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A5" s="9">
-        <v>1.2E-2</v>
+        <v>6.8999999999999903E-3</v>
       </c>
       <c r="B5" s="9">
         <v>5.1000000000000004E-3</v>
@@ -1501,12 +1496,12 @@
       </c>
       <c r="U5" t="str">
         <f ca="1">variablesVerzeichnis</f>
-        <v>unterverz/unterunterverz/20250708</v>
+        <v>unterverz/unterunterverz/20251218</v>
       </c>
     </row>
     <row r="6" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A6" s="9">
-        <v>0.5</v>
+        <v>0.28749999999999898</v>
       </c>
       <c r="B6" s="9">
         <v>0.21249999999999999</v>
@@ -1563,12 +1558,12 @@
       </c>
       <c r="U6" t="str">
         <f ca="1">variablesVerzeichnis</f>
-        <v>unterverz/unterunterverz/20250708</v>
+        <v>unterverz/unterunterverz/20251218</v>
       </c>
     </row>
     <row r="7" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A7" s="9">
-        <v>1.44E-2</v>
+        <v>8.8999999999999895E-3</v>
       </c>
       <c r="B7" s="9">
         <v>5.4999999999999997E-3</v>
@@ -1598,7 +1593,7 @@
     </row>
     <row r="8" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A8" s="9">
-        <v>0.02</v>
+        <v>1.1499999999999899E-2</v>
       </c>
       <c r="B8" s="9">
         <v>8.5000000000000006E-3</v>
@@ -1627,12 +1622,12 @@
       <c r="M8" s="3"/>
       <c r="U8" s="11" t="str">
         <f ca="1">"unterverz/unterunterverz/"&amp;TEXT(TODAY(),"JJJJMMTT")</f>
-        <v>unterverz/unterunterverz/20250708</v>
+        <v>unterverz/unterunterverz/20251218</v>
       </c>
     </row>
     <row r="9" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A9" s="9">
-        <v>2.8000000000000001E-2</v>
+        <v>1.6099999999999899E-2</v>
       </c>
       <c r="B9" s="9">
         <v>1.1900000000000001E-2</v>
@@ -1662,7 +1657,7 @@
     </row>
     <row r="10" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A10" s="9">
-        <v>5.4100000000000002E-2</v>
+        <v>3.1099999999999899E-2</v>
       </c>
       <c r="B10" s="9">
         <v>2.3E-2</v>
@@ -1692,7 +1687,7 @@
     </row>
     <row r="11" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A11" s="9">
-        <v>1.0176000000000001</v>
+        <v>0.63400000000000001</v>
       </c>
       <c r="B11" s="9">
         <v>0.3836</v>
@@ -1720,7 +1715,7 @@
       <c r="L11" s="3"/>
       <c r="M11" s="3"/>
       <c r="Q11" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="R11" s="17" t="s">
         <v>8</v>
@@ -1728,7 +1723,7 @@
     </row>
     <row r="12" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A12" s="9">
-        <v>0.91579999999999995</v>
+        <v>0.570599999999999</v>
       </c>
       <c r="B12" s="9">
         <v>0.34520000000000001</v>
@@ -1758,7 +1753,7 @@
     </row>
     <row r="13" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A13" s="9">
-        <v>3.85E-2</v>
+        <v>2.4E-2</v>
       </c>
       <c r="B13" s="9">
         <v>1.4500000000000001E-2</v>
@@ -1794,7 +1789,7 @@
     </row>
     <row r="14" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A14" s="9">
-        <v>3.85E-2</v>
+        <v>2.4E-2</v>
       </c>
       <c r="B14" s="9">
         <v>1.4500000000000001E-2</v>
@@ -1822,15 +1817,15 @@
       <c r="L14" s="3"/>
       <c r="M14" s="3"/>
       <c r="Q14" s="18" t="s">
+        <v>49</v>
+      </c>
+      <c r="R14" s="19" t="s">
         <v>50</v>
-      </c>
-      <c r="R14" s="19" t="s">
-        <v>51</v>
       </c>
     </row>
     <row r="15" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A15" s="9">
-        <v>2.4E-2</v>
+        <v>1.3799999999999899E-2</v>
       </c>
       <c r="B15" s="9">
         <v>1.0200000000000001E-2</v>
@@ -1867,7 +1862,7 @@
     </row>
     <row r="16" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A16" s="9">
-        <v>0.7</v>
+        <v>0.40250000000000002</v>
       </c>
       <c r="B16" s="9">
         <v>0.29749999999999999</v>
@@ -1899,12 +1894,12 @@
         <v>skipscript</v>
       </c>
       <c r="R16" s="2" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="17" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A17" s="9">
-        <v>0.7</v>
+        <v>0.40250000000000002</v>
       </c>
       <c r="B17" s="9">
         <v>0.29749999999999999</v>
@@ -1940,7 +1935,7 @@
     </row>
     <row r="18" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A18" s="9">
-        <v>2.0400000000000001E-2</v>
+        <v>1.2699999999999901E-2</v>
       </c>
       <c r="B18" s="9">
         <v>7.7000000000000002E-3</v>
@@ -1976,7 +1971,7 @@
     </row>
     <row r="19" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A19" s="9">
-        <v>2.0400000000000001E-2</v>
+        <v>1.2699999999999901E-2</v>
       </c>
       <c r="B19" s="9">
         <v>7.7000000000000002E-3</v>
@@ -2012,7 +2007,7 @@
     </row>
     <row r="20" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A20" s="9">
-        <v>2.8000000000000001E-2</v>
+        <v>1.6099999999999899E-2</v>
       </c>
       <c r="B20" s="9">
         <v>1.1900000000000001E-2</v>
@@ -2042,7 +2037,7 @@
     </row>
     <row r="21" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A21" s="9">
-        <v>0.04</v>
+        <v>2.2999999999999899E-2</v>
       </c>
       <c r="B21" s="9">
         <v>1.7000000000000001E-2</v>
@@ -2072,7 +2067,7 @@
     </row>
     <row r="22" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A22" s="9">
-        <v>4.4999999999999998E-2</v>
+        <v>2.5899999999999899E-2</v>
       </c>
       <c r="B22" s="9">
         <v>1.9099999999999999E-2</v>
@@ -2102,7 +2097,7 @@
     </row>
     <row r="23" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A23" s="9">
-        <v>0.1</v>
+        <v>5.7500000000000002E-2</v>
       </c>
       <c r="B23" s="9">
         <v>4.2500000000000003E-2</v>
@@ -2132,7 +2127,7 @@
     </row>
     <row r="24" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A24" s="9">
-        <v>9.01E-2</v>
+        <v>5.1799999999999902E-2</v>
       </c>
       <c r="B24" s="9">
         <v>3.8300000000000001E-2</v>
@@ -2162,7 +2157,7 @@
     </row>
     <row r="25" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A25" s="9">
-        <v>1.1803999999999999</v>
+        <v>0.73540000000000005</v>
       </c>
       <c r="B25" s="9">
         <v>0.44500000000000001</v>
@@ -2192,7 +2187,7 @@
     </row>
     <row r="26" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A26" s="9">
-        <v>0.875</v>
+        <v>0.54520000000000002</v>
       </c>
       <c r="B26" s="9">
         <v>0.32979999999999998</v>
@@ -2222,7 +2217,7 @@
     </row>
     <row r="27" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A27" s="9">
-        <v>0.95640000000000003</v>
+        <v>0.59589999999999899</v>
       </c>
       <c r="B27" s="9">
         <v>0.36049999999999999</v>
@@ -2252,7 +2247,7 @@
     </row>
     <row r="28" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A28" s="9">
-        <v>0.50880000000000003</v>
+        <v>0.317</v>
       </c>
       <c r="B28" s="9">
         <v>0.1918</v>
@@ -2282,7 +2277,7 @@
     </row>
     <row r="29" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A29" s="9">
-        <v>4.8899999999999999E-2</v>
+        <v>3.0499999999999899E-2</v>
       </c>
       <c r="B29" s="9">
         <v>1.84E-2</v>
@@ -2312,7 +2307,7 @@
     </row>
     <row r="30" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A30" s="9">
-        <v>3.3500000000000002E-2</v>
+        <v>2.0899999999999901E-2</v>
       </c>
       <c r="B30" s="9">
         <v>1.26E-2</v>
@@ -2342,7 +2337,7 @@
     </row>
     <row r="31" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A31" s="9">
-        <v>3.3500000000000002E-2</v>
+        <v>2.0899999999999901E-2</v>
       </c>
       <c r="B31" s="9">
         <v>1.26E-2</v>
@@ -2372,7 +2367,7 @@
     </row>
     <row r="32" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A32" s="9">
-        <v>2.0400000000000001E-2</v>
+        <v>1.2699999999999901E-2</v>
       </c>
       <c r="B32" s="9">
         <v>7.7000000000000002E-3</v>
@@ -2402,7 +2397,7 @@
     </row>
     <row r="33" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A33" s="9">
-        <v>0.8</v>
+        <v>0.46</v>
       </c>
       <c r="B33" s="9">
         <v>0.34</v>
@@ -2431,7 +2426,7 @@
     </row>
     <row r="34" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A34" s="9">
-        <v>0.6</v>
+        <v>0.34499999999999897</v>
       </c>
       <c r="B34" s="9">
         <v>0.255</v>
@@ -2459,7 +2454,7 @@
     </row>
     <row r="35" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A35" s="9">
-        <v>0.6</v>
+        <v>0.34499999999999897</v>
       </c>
       <c r="B35" s="9">
         <v>0.255</v>
@@ -2486,7 +2481,7 @@
     </row>
     <row r="36" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A36" s="9">
-        <v>0.2</v>
+        <v>0.115</v>
       </c>
       <c r="B36" s="9">
         <v>8.5000000000000006E-2</v>
@@ -2513,7 +2508,7 @@
     </row>
     <row r="37" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A37" s="9">
-        <v>3.0499999999999999E-2</v>
+        <v>1.8999999999999899E-2</v>
       </c>
       <c r="B37" s="9">
         <v>1.15E-2</v>
@@ -2540,7 +2535,7 @@
     </row>
     <row r="38" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A38" s="9">
-        <v>1.7399999999999999E-2</v>
+        <v>1.0800000000000001E-2</v>
       </c>
       <c r="B38" s="9">
         <v>6.6E-3</v>
@@ -2567,7 +2562,7 @@
     </row>
     <row r="39" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A39" s="9">
-        <v>1.7399999999999999E-2</v>
+        <v>1.0800000000000001E-2</v>
       </c>
       <c r="B39" s="9">
         <v>6.6E-3</v>
@@ -2594,7 +2589,7 @@
     </row>
     <row r="40" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A40" s="9">
-        <v>7.1000000000000004E-3</v>
+        <v>4.4000000000000003E-3</v>
       </c>
       <c r="B40" s="9">
         <v>2.7000000000000001E-3</v>
@@ -2621,7 +2616,7 @@
     </row>
     <row r="41" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A41" s="9">
-        <v>0.08</v>
+        <v>4.5999999999999902E-2</v>
       </c>
       <c r="B41" s="9">
         <v>3.4000000000000002E-2</v>
@@ -2648,7 +2643,7 @@
     </row>
     <row r="42" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A42" s="9">
-        <v>0.04</v>
+        <v>2.2999999999999899E-2</v>
       </c>
       <c r="B42" s="9">
         <v>1.7000000000000001E-2</v>
@@ -2675,7 +2670,7 @@
     </row>
     <row r="43" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A43" s="9">
-        <v>3.5000000000000003E-2</v>
+        <v>2.0099999999999899E-2</v>
       </c>
       <c r="B43" s="9">
         <v>1.49E-2</v>
@@ -2702,7 +2697,7 @@
     </row>
     <row r="44" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A44" s="9">
-        <v>0.02</v>
+        <v>1.1499999999999899E-2</v>
       </c>
       <c r="B44" s="9">
         <v>8.5000000000000006E-3</v>
@@ -2729,7 +2724,7 @@
     </row>
     <row r="45" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A45" s="9">
-        <v>0.14000000000000001</v>
+        <v>8.0500000000000002E-2</v>
       </c>
       <c r="B45" s="9">
         <v>5.9499999999999997E-2</v>
@@ -2756,7 +2751,7 @@
     </row>
     <row r="46" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A46" s="9">
-        <v>0.08</v>
+        <v>4.5999999999999902E-2</v>
       </c>
       <c r="B46" s="9">
         <v>3.4000000000000002E-2</v>
@@ -2783,7 +2778,7 @@
     </row>
     <row r="47" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A47" s="9">
-        <v>8.5000000000000006E-2</v>
+        <v>4.8899999999999902E-2</v>
       </c>
       <c r="B47" s="9">
         <v>3.61E-2</v>
@@ -2810,7 +2805,7 @@
     </row>
     <row r="48" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A48" s="9">
-        <v>0.04</v>
+        <v>2.2999999999999899E-2</v>
       </c>
       <c r="B48" s="9">
         <v>1.7000000000000001E-2</v>
@@ -2981,7 +2976,7 @@
     <row r="8" spans="1:8" x14ac:dyDescent="0.2">
       <c r="B8" s="7" t="str">
         <f ca="1">"  write.table(test_in[,1],file="""&amp;variablesVerzeichnis&amp;"/test_out.txt"",sep=""\t"",row.names=FALSE,col.names=FALSE,quote=FALSE)"</f>
-        <v xml:space="preserve">  write.table(test_in[,1],file="unterverz/unterunterverz/20250708/test_out.txt",sep="\t",row.names=FALSE,col.names=FALSE,quote=FALSE)</v>
+        <v xml:space="preserve">  write.table(test_in[,1],file="unterverz/unterunterverz/20251218/test_out.txt",sep="\t",row.names=FALSE,col.names=FALSE,quote=FALSE)</v>
       </c>
       <c r="C8"/>
       <c r="D8"/>
@@ -3015,7 +3010,7 @@
     <row r="11" spans="1:8" x14ac:dyDescent="0.2">
       <c r="B11" s="7" t="str">
         <f ca="1">"png(filename="""&amp;variablesVerzeichnis&amp;"/testdiagram.png"")"</f>
-        <v>png(filename="unterverz/unterunterverz/20250708/testdiagram.png")</v>
+        <v>png(filename="unterverz/unterunterverz/20251218/testdiagram.png")</v>
       </c>
       <c r="C11"/>
       <c r="D11"/>
@@ -3072,10 +3067,10 @@
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A16" s="18" t="s">
+        <v>49</v>
+      </c>
+      <c r="B16" s="19" t="s">
         <v>50</v>
-      </c>
-      <c r="B16" s="19" t="s">
-        <v>51</v>
       </c>
       <c r="C16"/>
       <c r="D16"/>
@@ -3121,7 +3116,7 @@
       </c>
       <c r="C19" t="str">
         <f ca="1">variablesVerzeichnis</f>
-        <v>unterverz/unterunterverz/20250708</v>
+        <v>unterverz/unterunterverz/20251218</v>
       </c>
       <c r="D19"/>
       <c r="E19"/>
@@ -3138,7 +3133,7 @@
       </c>
       <c r="C20" t="str">
         <f ca="1">variablesVerzeichnis</f>
-        <v>unterverz/unterunterverz/20250708</v>
+        <v>unterverz/unterunterverz/20251218</v>
       </c>
       <c r="D20"/>
       <c r="E20"/>
@@ -3171,10 +3166,10 @@
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A23" s="18" t="s">
+        <v>49</v>
+      </c>
+      <c r="B23" s="19" t="s">
         <v>50</v>
-      </c>
-      <c r="B23" s="19" t="s">
-        <v>51</v>
       </c>
       <c r="C23"/>
       <c r="D23" s="12"/>
@@ -9398,10 +9393,10 @@
       </c>
       <c r="I2" s="1"/>
       <c r="J2" s="18" t="s">
+        <v>49</v>
+      </c>
+      <c r="K2" s="19" t="s">
         <v>50</v>
-      </c>
-      <c r="K2" s="19" t="s">
-        <v>51</v>
       </c>
       <c r="L2"/>
     </row>
@@ -9512,13 +9507,13 @@
     <row r="9" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A9"/>
       <c r="J9" s="18" t="s">
+        <v>49</v>
+      </c>
+      <c r="K9" s="19" t="s">
         <v>50</v>
       </c>
-      <c r="K9" s="19" t="s">
-        <v>51</v>
-      </c>
       <c r="L9" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="O9" s="3"/>
       <c r="P9" s="2"/>
@@ -9703,18 +9698,18 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2" s="18" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B2" s="19" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" ht="242.25" x14ac:dyDescent="0.2">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" ht="318.75" x14ac:dyDescent="0.2">
       <c r="A3" s="3" t="s">
         <v>36</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>47</v>
+        <v>59</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">
@@ -9765,10 +9760,10 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2" s="18" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B2" s="19" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="395.25" x14ac:dyDescent="0.2">
@@ -9776,7 +9771,7 @@
         <v>36</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">
@@ -9830,10 +9825,10 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2" s="18" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B2" s="19" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="293.25" x14ac:dyDescent="0.2">
@@ -9841,7 +9836,7 @@
         <v>36</v>
       </c>
       <c r="B3" s="15" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">
@@ -9884,10 +9879,10 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2" s="18" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B2" s="19" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="89.25" x14ac:dyDescent="0.2">
@@ -9895,7 +9890,7 @@
         <v>36</v>
       </c>
       <c r="B3" s="16" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">

</xml_diff>